<commit_message>
Format Excel report for readability
</commit_message>
<xml_diff>
--- a/reports/gym_business_report.xlsx
+++ b/reports/gym_business_report.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Referral Sources" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Cancellation Rates" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Low Attendance Risk" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Business Insights" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,13 +22,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -50,8 +54,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,14 +426,18 @@
   </sheetPr>
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -505,16 +516,20 @@
   </sheetPr>
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>membership_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>monthly_fee</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Membership Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Estimated Monthly Revenue</t>
         </is>
       </c>
     </row>
@@ -571,16 +586,20 @@
   </sheetPr>
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>referral_source</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>member_count</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Referral Source</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Member Count</t>
         </is>
       </c>
     </row>
@@ -647,16 +666,20 @@
   </sheetPr>
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>membership_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>cancellation_rate</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Membership Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Cancellation Rate (%)</t>
         </is>
       </c>
     </row>
@@ -713,36 +736,44 @@
   </sheetPr>
   <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>member_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>membership_type</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>monthly_fee</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>sessions_attended</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>referral_source</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>cancelled</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Member ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Membership Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Monthly Fee</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Sessions Attended</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Referral Source</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Cancelled</t>
         </is>
       </c>
     </row>
@@ -1608,6 +1639,58 @@
       </c>
       <c r="F37" t="b">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Business Insights</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>The highest revenue membership type is Family with $3419.62 in estimated monthly revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>The strongest referral source is Walk-in with 68 members.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>The membership type with the highest cancellation rate is Family at 43.28%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>There are 36 members flagged as low-attendance risk.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add charts to business report
</commit_message>
<xml_diff>
--- a/reports/gym_business_report.xlsx
+++ b/reports/gym_business_report.xlsx
@@ -133,6 +133,423 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Revenue by Membership Type</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Revenue by Membership'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Revenue by Membership'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Revenue by Membership'!$B$2:$B$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Value</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Members by Referral Source</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Referral Sources'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Referral Sources'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Referral Sources'!$B$2:$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Value</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cancellation Rate by Membership Type</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Cancellation Rates'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Cancellation Rates'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cancellation Rates'!$B$2:$B$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Value</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -575,6 +992,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -655,6 +1073,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -725,6 +1144,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>